<commit_message>
projects/114-eudr-scope-mcp: every review finding fixed
A date written inside a consolidated entry is kept as its start date; an
amendment refresh cannot parse makes Annex answers say unverified (refresh
exits 1 then, 2 when it writes nothing); entries with exceptions are
partial (Chapters 47-48); corrigenda looked up for every act applied;
territories follow one rule; licence labelled per dataset (consolidated
text CC BY 4.0, OJ texts under the EUR-Lex re-use terms, Commission acts
also Decision 2011/833/EU). Tests: 106 -> 117.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017sPsTdJzLs7FzVt4vnAKxT
</commit_message>
<xml_diff>
--- a/projects/107-cbam-mcp/tests/fixtures/default_values_trimmed.xlsx
+++ b/projects/107-cbam-mcp/tests/fixtures/default_values_trimmed.xlsx
@@ -5,10 +5,12 @@
     <sheet name="Overview" sheetId="1" r:id="rId1"/>
     <sheet name="Version History" sheetId="2" r:id="rId2"/>
     <sheet name="Albania" sheetId="3" r:id="rId3"/>
-    <sheet name="India" sheetId="4" r:id="rId4"/>
-    <sheet name="Türkiye" sheetId="5" r:id="rId5"/>
-    <sheet name="_Other Countries and Territorie" sheetId="6" r:id="rId6"/>
-    <sheet name="Annex IV" sheetId="7" r:id="rId7"/>
+    <sheet name="Congo" sheetId="4" r:id="rId4"/>
+    <sheet name="Congo, Democratic Republic of" sheetId="5" r:id="rId5"/>
+    <sheet name="India" sheetId="6" r:id="rId6"/>
+    <sheet name="Türkiye" sheetId="7" r:id="rId7"/>
+    <sheet name="_Other Countries and Territorie" sheetId="8" r:id="rId8"/>
+    <sheet name="Annex IV" sheetId="9" r:id="rId9"/>
   </sheets>
 </workbook>
 </file>
@@ -104,6 +106,48 @@
     <t xml:space="preserve">White Portland cement</t>
   </si>
   <si>
+    <t xml:space="preserve">2523 29 00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Grey Portland cement</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0,900</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0,030</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0,930</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fertilisers</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3105</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mineral or chemical fertilisers containing two or three of the fertilising elements nitrogen, phosphorus and potassium</t>
+  </si>
+  <si>
+    <t xml:space="preserve">see below</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3105 10 00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mineral or chemical fertilisers of animal or vegetable origin, in tablets or similar forms, or in packages with a gross weight of &lt;= 10 kg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0,800</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0,060</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0,860</t>
+  </si>
+  <si>
     <t xml:space="preserve">Hydrogen</t>
   </si>
   <si>
@@ -116,15 +160,42 @@
     <t xml:space="preserve">N/A</t>
   </si>
   <si>
+    <t xml:space="preserve">Congo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0,850</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0,040</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0,890</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0,070</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10,820</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Congo, Democratic Republic of</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1,240</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1,250</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0,010</t>
+  </si>
+  <si>
     <t xml:space="preserve">India</t>
   </si>
   <si>
     <t xml:space="preserve">1,350</t>
   </si>
   <si>
-    <t xml:space="preserve">0,070</t>
-  </si>
-  <si>
     <t xml:space="preserve">1,410</t>
   </si>
   <si>
@@ -149,6 +220,18 @@
     <t xml:space="preserve">1,470</t>
   </si>
   <si>
+    <t xml:space="preserve">0,090</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1,480</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0,120</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0,980</t>
+  </si>
+  <si>
     <t xml:space="preserve">Aluminium</t>
   </si>
   <si>
@@ -203,9 +286,6 @@
     <t xml:space="preserve">Iron and non-alloy steel in ingots or other primary forms (excl. remelting scrap ingots, products obtained by continuous casting and iron of heading 7203)</t>
   </si>
   <si>
-    <t xml:space="preserve">see below</t>
-  </si>
-  <si>
     <t xml:space="preserve">7206 10 00</t>
   </si>
   <si>
@@ -242,15 +322,9 @@
     <t xml:space="preserve">2,674</t>
   </si>
   <si>
-    <t xml:space="preserve">10,820</t>
-  </si>
-  <si>
     <t xml:space="preserve">0,180</t>
   </si>
   <si>
-    <t xml:space="preserve">0,030</t>
-  </si>
-  <si>
     <t xml:space="preserve">0,210</t>
   </si>
   <si>
@@ -269,9 +343,6 @@
     <t xml:space="preserve">1,320</t>
   </si>
   <si>
-    <t xml:space="preserve">0,060</t>
-  </si>
-  <si>
     <t xml:space="preserve">1,370</t>
   </si>
   <si>
@@ -281,6 +352,18 @@
     <t xml:space="preserve">1,450</t>
   </si>
   <si>
+    <t xml:space="preserve">1,360</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0,080</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0,100</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1,000</t>
+  </si>
+  <si>
     <t xml:space="preserve">2,203</t>
   </si>
   <si>
@@ -311,7 +394,10 @@
     <t xml:space="preserve">0,320</t>
   </si>
   <si>
-    <t xml:space="preserve">1,480</t>
+    <t xml:space="preserve">1,490</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1,310</t>
   </si>
   <si>
     <t xml:space="preserve">3,198</t>
@@ -539,9 +625,89 @@
         <v>9</v>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="s">
+        <v>29</v>
+      </c>
+      <c r="B8" t="s">
+        <v>30</v>
+      </c>
+      <c r="C8" t="s">
+        <v>31</v>
+      </c>
+      <c r="D8" t="s">
+        <v>32</v>
+      </c>
+      <c r="E8" t="s">
+        <v>33</v>
+      </c>
+      <c r="F8" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="s">
+        <v>34</v>
+      </c>
+      <c r="B12" t="s">
+        <v>9</v>
+      </c>
+      <c r="C12" t="s">
+        <v>9</v>
+      </c>
+      <c r="D12" t="s">
+        <v>9</v>
+      </c>
+      <c r="E12" t="s">
+        <v>9</v>
+      </c>
+      <c r="F12" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="s">
+        <v>35</v>
+      </c>
+      <c r="B32" t="s">
+        <v>36</v>
+      </c>
+      <c r="C32" t="s">
+        <v>37</v>
+      </c>
+      <c r="D32" t="s">
+        <v>37</v>
+      </c>
+      <c r="E32" t="s">
+        <v>37</v>
+      </c>
+      <c r="F32" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="s">
+        <v>38</v>
+      </c>
+      <c r="B33" t="s">
+        <v>39</v>
+      </c>
+      <c r="C33" t="s">
+        <v>40</v>
+      </c>
+      <c r="D33" t="s">
+        <v>41</v>
+      </c>
+      <c r="E33" t="s">
+        <v>42</v>
+      </c>
+      <c r="F33" t="s">
+        <v>9</v>
+      </c>
+    </row>
     <row r="42">
       <c r="A42" t="s">
-        <v>29</v>
+        <v>43</v>
       </c>
       <c r="B42" t="s">
         <v>9</v>
@@ -561,19 +727,19 @@
     </row>
     <row r="43">
       <c r="A43" t="s">
-        <v>30</v>
+        <v>44</v>
       </c>
       <c r="B43" t="s">
-        <v>29</v>
+        <v>43</v>
       </c>
       <c r="C43" t="s">
-        <v>31</v>
+        <v>45</v>
       </c>
       <c r="D43" t="s">
-        <v>32</v>
+        <v>46</v>
       </c>
       <c r="E43" t="s">
-        <v>31</v>
+        <v>45</v>
       </c>
       <c r="F43" t="s">
         <v>9</v>
@@ -588,7 +754,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>33</v>
+        <v>47</v>
       </c>
       <c r="B1" t="s">
         <v>9</v>
@@ -674,16 +840,16 @@
         <v>21</v>
       </c>
       <c r="C5" t="s">
-        <v>34</v>
+        <v>19</v>
       </c>
       <c r="D5" t="s">
-        <v>35</v>
+        <v>19</v>
       </c>
       <c r="E5" t="s">
-        <v>36</v>
+        <v>19</v>
       </c>
       <c r="F5" t="s">
-        <v>37</v>
+        <v>9</v>
       </c>
     </row>
     <row r="6">
@@ -694,13 +860,13 @@
         <v>23</v>
       </c>
       <c r="C6" t="s">
-        <v>38</v>
+        <v>48</v>
       </c>
       <c r="D6" t="s">
-        <v>39</v>
+        <v>49</v>
       </c>
       <c r="E6" t="s">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="F6" t="s">
         <v>26</v>
@@ -714,276 +880,76 @@
         <v>28</v>
       </c>
       <c r="C7" t="s">
-        <v>41</v>
+        <v>19</v>
       </c>
       <c r="D7" t="s">
-        <v>42</v>
+        <v>19</v>
       </c>
       <c r="E7" t="s">
+        <v>19</v>
+      </c>
+      <c r="F7" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s">
+        <v>29</v>
+      </c>
+      <c r="B8" t="s">
+        <v>30</v>
+      </c>
+      <c r="C8" t="s">
+        <v>48</v>
+      </c>
+      <c r="D8" t="s">
+        <v>51</v>
+      </c>
+      <c r="E8" t="s">
+        <v>33</v>
+      </c>
+      <c r="F8" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="s">
         <v>43</v>
       </c>
-      <c r="F7" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="s">
+      <c r="B12" t="s">
+        <v>9</v>
+      </c>
+      <c r="C12" t="s">
+        <v>9</v>
+      </c>
+      <c r="D12" t="s">
+        <v>9</v>
+      </c>
+      <c r="E12" t="s">
+        <v>9</v>
+      </c>
+      <c r="F12" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="s">
         <v>44</v>
       </c>
-      <c r="B42" t="s">
-        <v>9</v>
-      </c>
-      <c r="C42" t="s">
-        <v>9</v>
-      </c>
-      <c r="D42" t="s">
-        <v>9</v>
-      </c>
-      <c r="E42" t="s">
-        <v>9</v>
-      </c>
-      <c r="F42" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="s">
-        <v>45</v>
-      </c>
-      <c r="B43" t="s">
+      <c r="B13" t="s">
+        <v>43</v>
+      </c>
+      <c r="C13" t="s">
+        <v>52</v>
+      </c>
+      <c r="D13" t="s">
         <v>46</v>
       </c>
-      <c r="C43" t="s">
-        <v>47</v>
-      </c>
-      <c r="D43" t="s">
-        <v>32</v>
-      </c>
-      <c r="E43" t="s">
-        <v>47</v>
-      </c>
-      <c r="F43" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" t="s">
-        <v>49</v>
-      </c>
-      <c r="B56" t="s">
-        <v>50</v>
-      </c>
-      <c r="C56" t="s">
-        <v>51</v>
-      </c>
-      <c r="D56" t="s">
-        <v>32</v>
-      </c>
-      <c r="E56" t="s">
-        <v>51</v>
-      </c>
-      <c r="F56" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" t="s">
+      <c r="E13" t="s">
         <v>52</v>
       </c>
-      <c r="B57" t="s">
-        <v>53</v>
-      </c>
-      <c r="C57" t="s">
-        <v>51</v>
-      </c>
-      <c r="D57" t="s">
-        <v>32</v>
-      </c>
-      <c r="E57" t="s">
-        <v>51</v>
-      </c>
-      <c r="F57" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" t="s">
-        <v>54</v>
-      </c>
-      <c r="B58" t="s">
-        <v>50</v>
-      </c>
-      <c r="C58" t="s">
-        <v>51</v>
-      </c>
-      <c r="D58" t="s">
-        <v>32</v>
-      </c>
-      <c r="E58" t="s">
-        <v>51</v>
-      </c>
-      <c r="F58" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" t="s">
-        <v>29</v>
-      </c>
-      <c r="B67" t="s">
-        <v>9</v>
-      </c>
-      <c r="C67" t="s">
-        <v>9</v>
-      </c>
-      <c r="D67" t="s">
-        <v>9</v>
-      </c>
-      <c r="E67" t="s">
-        <v>9</v>
-      </c>
-      <c r="F67" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" t="s">
-        <v>30</v>
-      </c>
-      <c r="B68" t="s">
-        <v>29</v>
-      </c>
-      <c r="C68" t="s">
-        <v>31</v>
-      </c>
-      <c r="D68" t="s">
-        <v>32</v>
-      </c>
-      <c r="E68" t="s">
-        <v>31</v>
-      </c>
-      <c r="F68" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" t="s">
-        <v>55</v>
-      </c>
-      <c r="B69" t="s">
-        <v>9</v>
-      </c>
-      <c r="C69" t="s">
-        <v>9</v>
-      </c>
-      <c r="D69" t="s">
-        <v>9</v>
-      </c>
-      <c r="E69" t="s">
-        <v>9</v>
-      </c>
-      <c r="F69" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" t="s">
-        <v>56</v>
-      </c>
-      <c r="B70" t="s">
-        <v>57</v>
-      </c>
-      <c r="C70" t="s">
-        <v>58</v>
-      </c>
-      <c r="D70" t="s">
-        <v>39</v>
-      </c>
-      <c r="E70" t="s">
-        <v>59</v>
-      </c>
-      <c r="F70" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="79">
-      <c r="A79" t="s">
-        <v>60</v>
-      </c>
-      <c r="B79" t="s">
-        <v>61</v>
-      </c>
-      <c r="C79" t="s">
-        <v>62</v>
-      </c>
-      <c r="D79" t="s">
-        <v>62</v>
-      </c>
-      <c r="E79" t="s">
-        <v>62</v>
-      </c>
-      <c r="F79" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="80">
-      <c r="A80" t="s">
-        <v>63</v>
-      </c>
-      <c r="B80" t="s">
-        <v>64</v>
-      </c>
-      <c r="C80" t="s">
-        <v>65</v>
-      </c>
-      <c r="D80" t="s">
-        <v>32</v>
-      </c>
-      <c r="E80" t="s">
-        <v>65</v>
-      </c>
-      <c r="F80" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="81">
-      <c r="A81" t="s">
-        <v>67</v>
-      </c>
-      <c r="B81" t="s">
-        <v>68</v>
-      </c>
-      <c r="C81" t="s">
-        <v>65</v>
-      </c>
-      <c r="D81" t="s">
-        <v>32</v>
-      </c>
-      <c r="E81" t="s">
-        <v>65</v>
-      </c>
-      <c r="F81" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="101">
-      <c r="A101" t="s">
-        <v>69</v>
-      </c>
-      <c r="B101" t="s">
-        <v>70</v>
-      </c>
-      <c r="C101" t="s">
-        <v>71</v>
-      </c>
-      <c r="D101" t="s">
-        <v>32</v>
-      </c>
-      <c r="E101" t="s">
-        <v>71</v>
-      </c>
-      <c r="F101" t="s">
-        <v>66</v>
+      <c r="F13" t="s">
+        <v>9</v>
       </c>
     </row>
   </sheetData>
@@ -995,7 +961,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>72</v>
+        <v>53</v>
       </c>
       <c r="B1" t="s">
         <v>9</v>
@@ -1101,16 +1067,16 @@
         <v>23</v>
       </c>
       <c r="C6" t="s">
-        <v>19</v>
+        <v>54</v>
       </c>
       <c r="D6" t="s">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="E6" t="s">
-        <v>19</v>
+        <v>55</v>
       </c>
       <c r="F6" t="s">
-        <v>9</v>
+        <v>26</v>
       </c>
     </row>
     <row r="7">
@@ -1133,264 +1099,24 @@
         <v>9</v>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" t="s">
-        <v>44</v>
-      </c>
-      <c r="B42" t="s">
-        <v>9</v>
-      </c>
-      <c r="C42" t="s">
-        <v>9</v>
-      </c>
-      <c r="D42" t="s">
-        <v>9</v>
-      </c>
-      <c r="E42" t="s">
-        <v>9</v>
-      </c>
-      <c r="F42" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="s">
-        <v>45</v>
-      </c>
-      <c r="B43" t="s">
-        <v>46</v>
-      </c>
-      <c r="C43" t="s">
-        <v>73</v>
-      </c>
-      <c r="D43" t="s">
-        <v>32</v>
-      </c>
-      <c r="E43" t="s">
-        <v>73</v>
-      </c>
-      <c r="F43" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" t="s">
-        <v>49</v>
-      </c>
-      <c r="B56" t="s">
-        <v>50</v>
-      </c>
-      <c r="C56" t="s">
-        <v>74</v>
-      </c>
-      <c r="D56" t="s">
-        <v>32</v>
-      </c>
-      <c r="E56" t="s">
-        <v>74</v>
-      </c>
-      <c r="F56" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" t="s">
-        <v>52</v>
-      </c>
-      <c r="B57" t="s">
-        <v>53</v>
-      </c>
-      <c r="C57" t="s">
-        <v>74</v>
-      </c>
-      <c r="D57" t="s">
-        <v>32</v>
-      </c>
-      <c r="E57" t="s">
-        <v>74</v>
-      </c>
-      <c r="F57" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" t="s">
+    <row r="8">
+      <c r="A8" t="s">
+        <v>29</v>
+      </c>
+      <c r="B8" t="s">
+        <v>30</v>
+      </c>
+      <c r="C8" t="s">
         <v>54</v>
       </c>
-      <c r="B58" t="s">
-        <v>50</v>
-      </c>
-      <c r="C58" t="s">
-        <v>74</v>
-      </c>
-      <c r="D58" t="s">
-        <v>32</v>
-      </c>
-      <c r="E58" t="s">
-        <v>74</v>
-      </c>
-      <c r="F58" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" t="s">
-        <v>29</v>
-      </c>
-      <c r="B67" t="s">
-        <v>9</v>
-      </c>
-      <c r="C67" t="s">
-        <v>9</v>
-      </c>
-      <c r="D67" t="s">
-        <v>9</v>
-      </c>
-      <c r="E67" t="s">
-        <v>9</v>
-      </c>
-      <c r="F67" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" t="s">
-        <v>30</v>
-      </c>
-      <c r="B68" t="s">
-        <v>29</v>
-      </c>
-      <c r="C68" t="s">
-        <v>75</v>
-      </c>
-      <c r="D68" t="s">
-        <v>32</v>
-      </c>
-      <c r="E68" t="s">
-        <v>75</v>
-      </c>
-      <c r="F68" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" t="s">
+      <c r="D8" t="s">
+        <v>56</v>
+      </c>
+      <c r="E8" t="s">
         <v>55</v>
       </c>
-      <c r="B69" t="s">
-        <v>9</v>
-      </c>
-      <c r="C69" t="s">
-        <v>9</v>
-      </c>
-      <c r="D69" t="s">
-        <v>9</v>
-      </c>
-      <c r="E69" t="s">
-        <v>9</v>
-      </c>
-      <c r="F69" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" t="s">
-        <v>56</v>
-      </c>
-      <c r="B70" t="s">
-        <v>57</v>
-      </c>
-      <c r="C70" t="s">
-        <v>76</v>
-      </c>
-      <c r="D70" t="s">
-        <v>77</v>
-      </c>
-      <c r="E70" t="s">
-        <v>78</v>
-      </c>
-      <c r="F70" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="79">
-      <c r="A79" t="s">
-        <v>60</v>
-      </c>
-      <c r="B79" t="s">
-        <v>61</v>
-      </c>
-      <c r="C79" t="s">
-        <v>62</v>
-      </c>
-      <c r="D79" t="s">
-        <v>62</v>
-      </c>
-      <c r="E79" t="s">
-        <v>62</v>
-      </c>
-      <c r="F79" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="80">
-      <c r="A80" t="s">
-        <v>63</v>
-      </c>
-      <c r="B80" t="s">
-        <v>64</v>
-      </c>
-      <c r="C80" t="s">
-        <v>79</v>
-      </c>
-      <c r="D80" t="s">
-        <v>32</v>
-      </c>
-      <c r="E80" t="s">
-        <v>79</v>
-      </c>
-      <c r="F80" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="81">
-      <c r="A81" t="s">
-        <v>67</v>
-      </c>
-      <c r="B81" t="s">
-        <v>68</v>
-      </c>
-      <c r="C81" t="s">
-        <v>79</v>
-      </c>
-      <c r="D81" t="s">
-        <v>32</v>
-      </c>
-      <c r="E81" t="s">
-        <v>79</v>
-      </c>
-      <c r="F81" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="101">
-      <c r="A101" t="s">
-        <v>69</v>
-      </c>
-      <c r="B101" t="s">
-        <v>70</v>
-      </c>
-      <c r="C101" t="s">
-        <v>80</v>
-      </c>
-      <c r="D101" t="s">
-        <v>32</v>
-      </c>
-      <c r="E101" t="s">
-        <v>80</v>
-      </c>
-      <c r="F101" t="s">
-        <v>66</v>
+      <c r="F8" t="s">
+        <v>9</v>
       </c>
     </row>
   </sheetData>
@@ -1402,7 +1128,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>81</v>
+        <v>57</v>
       </c>
       <c r="B1" t="s">
         <v>9</v>
@@ -1468,13 +1194,13 @@
         <v>18</v>
       </c>
       <c r="C4" t="s">
-        <v>78</v>
+        <v>19</v>
       </c>
       <c r="D4" t="s">
-        <v>35</v>
+        <v>19</v>
       </c>
       <c r="E4" t="s">
-        <v>82</v>
+        <v>19</v>
       </c>
       <c r="F4" t="s">
         <v>9</v>
@@ -1488,16 +1214,16 @@
         <v>21</v>
       </c>
       <c r="C5" t="s">
-        <v>83</v>
+        <v>58</v>
       </c>
       <c r="D5" t="s">
-        <v>84</v>
+        <v>51</v>
       </c>
       <c r="E5" t="s">
-        <v>85</v>
+        <v>59</v>
       </c>
       <c r="F5" t="s">
-        <v>37</v>
+        <v>60</v>
       </c>
     </row>
     <row r="6">
@@ -1508,13 +1234,13 @@
         <v>23</v>
       </c>
       <c r="C6" t="s">
-        <v>85</v>
+        <v>61</v>
       </c>
       <c r="D6" t="s">
-        <v>39</v>
+        <v>62</v>
       </c>
       <c r="E6" t="s">
-        <v>36</v>
+        <v>63</v>
       </c>
       <c r="F6" t="s">
         <v>26</v>
@@ -1528,21 +1254,101 @@
         <v>28</v>
       </c>
       <c r="C7" t="s">
-        <v>86</v>
+        <v>64</v>
       </c>
       <c r="D7" t="s">
-        <v>42</v>
+        <v>65</v>
       </c>
       <c r="E7" t="s">
-        <v>87</v>
+        <v>66</v>
       </c>
       <c r="F7" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s">
+        <v>29</v>
+      </c>
+      <c r="B8" t="s">
+        <v>30</v>
+      </c>
+      <c r="C8" t="s">
+        <v>61</v>
+      </c>
+      <c r="D8" t="s">
+        <v>67</v>
+      </c>
+      <c r="E8" t="s">
+        <v>68</v>
+      </c>
+      <c r="F8" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="s">
+        <v>34</v>
+      </c>
+      <c r="B12" t="s">
+        <v>9</v>
+      </c>
+      <c r="C12" t="s">
+        <v>9</v>
+      </c>
+      <c r="D12" t="s">
+        <v>9</v>
+      </c>
+      <c r="E12" t="s">
+        <v>9</v>
+      </c>
+      <c r="F12" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="s">
+        <v>35</v>
+      </c>
+      <c r="B32" t="s">
+        <v>36</v>
+      </c>
+      <c r="C32" t="s">
+        <v>37</v>
+      </c>
+      <c r="D32" t="s">
+        <v>37</v>
+      </c>
+      <c r="E32" t="s">
+        <v>37</v>
+      </c>
+      <c r="F32" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="s">
+        <v>38</v>
+      </c>
+      <c r="B33" t="s">
+        <v>39</v>
+      </c>
+      <c r="C33" t="s">
+        <v>48</v>
+      </c>
+      <c r="D33" t="s">
+        <v>69</v>
+      </c>
+      <c r="E33" t="s">
+        <v>70</v>
+      </c>
+      <c r="F33" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="s">
-        <v>44</v>
+        <v>71</v>
       </c>
       <c r="B42" t="s">
         <v>9</v>
@@ -1562,87 +1368,87 @@
     </row>
     <row r="43">
       <c r="A43" t="s">
-        <v>45</v>
+        <v>72</v>
       </c>
       <c r="B43" t="s">
+        <v>73</v>
+      </c>
+      <c r="C43" t="s">
+        <v>74</v>
+      </c>
+      <c r="D43" t="s">
         <v>46</v>
       </c>
-      <c r="C43" t="s">
-        <v>88</v>
-      </c>
-      <c r="D43" t="s">
-        <v>32</v>
-      </c>
       <c r="E43" t="s">
-        <v>88</v>
+        <v>74</v>
       </c>
       <c r="F43" t="s">
-        <v>48</v>
+        <v>75</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="s">
-        <v>49</v>
+        <v>76</v>
       </c>
       <c r="B56" t="s">
-        <v>50</v>
+        <v>77</v>
       </c>
       <c r="C56" t="s">
-        <v>89</v>
+        <v>78</v>
       </c>
       <c r="D56" t="s">
-        <v>32</v>
+        <v>46</v>
       </c>
       <c r="E56" t="s">
-        <v>89</v>
+        <v>78</v>
       </c>
       <c r="F56" t="s">
-        <v>48</v>
+        <v>75</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="s">
-        <v>52</v>
+        <v>79</v>
       </c>
       <c r="B57" t="s">
-        <v>53</v>
+        <v>80</v>
       </c>
       <c r="C57" t="s">
-        <v>89</v>
+        <v>78</v>
       </c>
       <c r="D57" t="s">
-        <v>32</v>
+        <v>46</v>
       </c>
       <c r="E57" t="s">
-        <v>89</v>
+        <v>78</v>
       </c>
       <c r="F57" t="s">
-        <v>48</v>
+        <v>75</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="s">
-        <v>54</v>
+        <v>81</v>
       </c>
       <c r="B58" t="s">
-        <v>50</v>
+        <v>77</v>
       </c>
       <c r="C58" t="s">
-        <v>89</v>
+        <v>78</v>
       </c>
       <c r="D58" t="s">
-        <v>32</v>
+        <v>46</v>
       </c>
       <c r="E58" t="s">
-        <v>89</v>
+        <v>78</v>
       </c>
       <c r="F58" t="s">
-        <v>48</v>
+        <v>75</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="s">
-        <v>29</v>
+        <v>43</v>
       </c>
       <c r="B67" t="s">
         <v>9</v>
@@ -1662,19 +1468,19 @@
     </row>
     <row r="68">
       <c r="A68" t="s">
-        <v>30</v>
+        <v>44</v>
       </c>
       <c r="B68" t="s">
-        <v>29</v>
+        <v>43</v>
       </c>
       <c r="C68" t="s">
-        <v>90</v>
+        <v>45</v>
       </c>
       <c r="D68" t="s">
-        <v>32</v>
+        <v>46</v>
       </c>
       <c r="E68" t="s">
-        <v>90</v>
+        <v>45</v>
       </c>
       <c r="F68" t="s">
         <v>9</v>
@@ -1682,7 +1488,7 @@
     </row>
     <row r="69">
       <c r="A69" t="s">
-        <v>55</v>
+        <v>82</v>
       </c>
       <c r="B69" t="s">
         <v>9</v>
@@ -1702,19 +1508,19 @@
     </row>
     <row r="70">
       <c r="A70" t="s">
-        <v>56</v>
+        <v>83</v>
       </c>
       <c r="B70" t="s">
-        <v>57</v>
+        <v>84</v>
       </c>
       <c r="C70" t="s">
-        <v>91</v>
+        <v>85</v>
       </c>
       <c r="D70" t="s">
-        <v>35</v>
+        <v>62</v>
       </c>
       <c r="E70" t="s">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="F70" t="s">
         <v>9</v>
@@ -1722,19 +1528,19 @@
     </row>
     <row r="79">
       <c r="A79" t="s">
-        <v>60</v>
+        <v>87</v>
       </c>
       <c r="B79" t="s">
-        <v>61</v>
+        <v>88</v>
       </c>
       <c r="C79" t="s">
-        <v>62</v>
+        <v>37</v>
       </c>
       <c r="D79" t="s">
-        <v>62</v>
+        <v>37</v>
       </c>
       <c r="E79" t="s">
-        <v>62</v>
+        <v>37</v>
       </c>
       <c r="F79" t="s">
         <v>9</v>
@@ -1742,62 +1548,62 @@
     </row>
     <row r="80">
       <c r="A80" t="s">
-        <v>63</v>
+        <v>89</v>
       </c>
       <c r="B80" t="s">
-        <v>64</v>
+        <v>90</v>
       </c>
       <c r="C80" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="D80" t="s">
-        <v>32</v>
+        <v>46</v>
       </c>
       <c r="E80" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="F80" t="s">
-        <v>66</v>
+        <v>92</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="s">
-        <v>67</v>
+        <v>93</v>
       </c>
       <c r="B81" t="s">
-        <v>68</v>
+        <v>94</v>
       </c>
       <c r="C81" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="D81" t="s">
-        <v>32</v>
+        <v>46</v>
       </c>
       <c r="E81" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="F81" t="s">
-        <v>66</v>
+        <v>92</v>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="s">
-        <v>69</v>
+        <v>95</v>
       </c>
       <c r="B101" t="s">
-        <v>70</v>
+        <v>96</v>
       </c>
       <c r="C101" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="D101" t="s">
-        <v>32</v>
+        <v>46</v>
       </c>
       <c r="E101" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="F101" t="s">
-        <v>66</v>
+        <v>92</v>
       </c>
     </row>
   </sheetData>
@@ -1809,7 +1615,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="B1" t="s">
         <v>9</v>
@@ -1818,6 +1624,12 @@
         <v>9</v>
       </c>
       <c r="D1" t="s">
+        <v>9</v>
+      </c>
+      <c r="E1" t="s">
+        <v>9</v>
+      </c>
+      <c r="F1" t="s">
         <v>9</v>
       </c>
     </row>
@@ -1829,9 +1641,15 @@
         <v>11</v>
       </c>
       <c r="C2" t="s">
-        <v>96</v>
+        <v>12</v>
       </c>
       <c r="D2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E2" t="s">
+        <v>14</v>
+      </c>
+      <c r="F2" t="s">
         <v>15</v>
       </c>
     </row>
@@ -1848,6 +1666,12 @@
       <c r="D3" t="s">
         <v>9</v>
       </c>
+      <c r="E3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F3" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
@@ -1857,9 +1681,15 @@
         <v>18</v>
       </c>
       <c r="C4" t="s">
-        <v>97</v>
+        <v>19</v>
       </c>
       <c r="D4" t="s">
+        <v>19</v>
+      </c>
+      <c r="E4" t="s">
+        <v>19</v>
+      </c>
+      <c r="F4" t="s">
         <v>9</v>
       </c>
     </row>
@@ -1871,10 +1701,16 @@
         <v>21</v>
       </c>
       <c r="C5" t="s">
-        <v>36</v>
+        <v>19</v>
       </c>
       <c r="D5" t="s">
-        <v>37</v>
+        <v>19</v>
+      </c>
+      <c r="E5" t="s">
+        <v>19</v>
+      </c>
+      <c r="F5" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="6">
@@ -1885,10 +1721,16 @@
         <v>23</v>
       </c>
       <c r="C6" t="s">
-        <v>40</v>
+        <v>19</v>
       </c>
       <c r="D6" t="s">
-        <v>26</v>
+        <v>19</v>
+      </c>
+      <c r="E6" t="s">
+        <v>19</v>
+      </c>
+      <c r="F6" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="7">
@@ -1899,15 +1741,101 @@
         <v>28</v>
       </c>
       <c r="C7" t="s">
-        <v>98</v>
+        <v>19</v>
       </c>
       <c r="D7" t="s">
+        <v>19</v>
+      </c>
+      <c r="E7" t="s">
+        <v>19</v>
+      </c>
+      <c r="F7" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s">
+        <v>29</v>
+      </c>
+      <c r="B8" t="s">
+        <v>30</v>
+      </c>
+      <c r="C8" t="s">
+        <v>19</v>
+      </c>
+      <c r="D8" t="s">
+        <v>19</v>
+      </c>
+      <c r="E8" t="s">
+        <v>19</v>
+      </c>
+      <c r="F8" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="s">
+        <v>34</v>
+      </c>
+      <c r="B12" t="s">
+        <v>9</v>
+      </c>
+      <c r="C12" t="s">
+        <v>9</v>
+      </c>
+      <c r="D12" t="s">
+        <v>9</v>
+      </c>
+      <c r="E12" t="s">
+        <v>9</v>
+      </c>
+      <c r="F12" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="s">
+        <v>35</v>
+      </c>
+      <c r="B32" t="s">
+        <v>36</v>
+      </c>
+      <c r="C32" t="s">
+        <v>37</v>
+      </c>
+      <c r="D32" t="s">
+        <v>37</v>
+      </c>
+      <c r="E32" t="s">
+        <v>37</v>
+      </c>
+      <c r="F32" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="s">
+        <v>38</v>
+      </c>
+      <c r="B33" t="s">
+        <v>39</v>
+      </c>
+      <c r="C33" t="s">
+        <v>40</v>
+      </c>
+      <c r="D33" t="s">
+        <v>41</v>
+      </c>
+      <c r="E33" t="s">
+        <v>42</v>
+      </c>
+      <c r="F33" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="s">
-        <v>44</v>
+        <v>71</v>
       </c>
       <c r="B42" t="s">
         <v>9</v>
@@ -1916,68 +1844,98 @@
         <v>9</v>
       </c>
       <c r="D42" t="s">
+        <v>9</v>
+      </c>
+      <c r="E42" t="s">
+        <v>9</v>
+      </c>
+      <c r="F42" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="s">
-        <v>45</v>
+        <v>72</v>
       </c>
       <c r="B43" t="s">
-        <v>46</v>
+        <v>73</v>
       </c>
       <c r="C43" t="s">
         <v>99</v>
       </c>
       <c r="D43" t="s">
-        <v>48</v>
+        <v>46</v>
+      </c>
+      <c r="E43" t="s">
+        <v>99</v>
+      </c>
+      <c r="F43" t="s">
+        <v>75</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="s">
-        <v>49</v>
+        <v>76</v>
       </c>
       <c r="B56" t="s">
-        <v>50</v>
+        <v>77</v>
       </c>
       <c r="C56" t="s">
         <v>100</v>
       </c>
       <c r="D56" t="s">
-        <v>48</v>
+        <v>46</v>
+      </c>
+      <c r="E56" t="s">
+        <v>100</v>
+      </c>
+      <c r="F56" t="s">
+        <v>75</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="s">
-        <v>52</v>
+        <v>79</v>
       </c>
       <c r="B57" t="s">
-        <v>53</v>
+        <v>80</v>
       </c>
       <c r="C57" t="s">
         <v>100</v>
       </c>
       <c r="D57" t="s">
-        <v>48</v>
+        <v>46</v>
+      </c>
+      <c r="E57" t="s">
+        <v>100</v>
+      </c>
+      <c r="F57" t="s">
+        <v>75</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="s">
-        <v>54</v>
+        <v>81</v>
       </c>
       <c r="B58" t="s">
-        <v>50</v>
+        <v>77</v>
       </c>
       <c r="C58" t="s">
         <v>100</v>
       </c>
       <c r="D58" t="s">
-        <v>48</v>
+        <v>46</v>
+      </c>
+      <c r="E58" t="s">
+        <v>100</v>
+      </c>
+      <c r="F58" t="s">
+        <v>75</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="s">
-        <v>29</v>
+        <v>43</v>
       </c>
       <c r="B67" t="s">
         <v>9</v>
@@ -1986,26 +1944,38 @@
         <v>9</v>
       </c>
       <c r="D67" t="s">
+        <v>9</v>
+      </c>
+      <c r="E67" t="s">
+        <v>9</v>
+      </c>
+      <c r="F67" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="s">
-        <v>30</v>
+        <v>44</v>
       </c>
       <c r="B68" t="s">
-        <v>29</v>
+        <v>43</v>
       </c>
       <c r="C68" t="s">
-        <v>101</v>
+        <v>52</v>
       </c>
       <c r="D68" t="s">
+        <v>46</v>
+      </c>
+      <c r="E68" t="s">
+        <v>52</v>
+      </c>
+      <c r="F68" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="s">
-        <v>55</v>
+        <v>82</v>
       </c>
       <c r="B69" t="s">
         <v>9</v>
@@ -2014,77 +1984,943 @@
         <v>9</v>
       </c>
       <c r="D69" t="s">
+        <v>9</v>
+      </c>
+      <c r="E69" t="s">
+        <v>9</v>
+      </c>
+      <c r="F69" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="s">
-        <v>56</v>
+        <v>83</v>
       </c>
       <c r="B70" t="s">
-        <v>57</v>
+        <v>84</v>
       </c>
       <c r="C70" t="s">
+        <v>101</v>
+      </c>
+      <c r="D70" t="s">
+        <v>32</v>
+      </c>
+      <c r="E70" t="s">
         <v>102</v>
       </c>
-      <c r="D70" t="s">
+      <c r="F70" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="s">
-        <v>60</v>
+        <v>87</v>
       </c>
       <c r="B79" t="s">
-        <v>61</v>
+        <v>88</v>
       </c>
       <c r="C79" t="s">
-        <v>62</v>
+        <v>37</v>
       </c>
       <c r="D79" t="s">
+        <v>37</v>
+      </c>
+      <c r="E79" t="s">
+        <v>37</v>
+      </c>
+      <c r="F79" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="s">
-        <v>63</v>
+        <v>89</v>
       </c>
       <c r="B80" t="s">
-        <v>64</v>
+        <v>90</v>
       </c>
       <c r="C80" t="s">
         <v>103</v>
       </c>
       <c r="D80" t="s">
-        <v>66</v>
+        <v>46</v>
+      </c>
+      <c r="E80" t="s">
+        <v>103</v>
+      </c>
+      <c r="F80" t="s">
+        <v>92</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="s">
-        <v>67</v>
+        <v>93</v>
       </c>
       <c r="B81" t="s">
-        <v>68</v>
+        <v>94</v>
       </c>
       <c r="C81" t="s">
         <v>103</v>
       </c>
       <c r="D81" t="s">
-        <v>66</v>
+        <v>46</v>
+      </c>
+      <c r="E81" t="s">
+        <v>103</v>
+      </c>
+      <c r="F81" t="s">
+        <v>92</v>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="s">
-        <v>69</v>
+        <v>95</v>
       </c>
       <c r="B101" t="s">
-        <v>70</v>
+        <v>96</v>
       </c>
       <c r="C101" t="s">
         <v>104</v>
       </c>
       <c r="D101" t="s">
-        <v>66</v>
+        <v>46</v>
+      </c>
+      <c r="E101" t="s">
+        <v>104</v>
+      </c>
+      <c r="F101" t="s">
+        <v>92</v>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>105</v>
+      </c>
+      <c r="B1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1" t="s">
+        <v>9</v>
+      </c>
+      <c r="E1" t="s">
+        <v>9</v>
+      </c>
+      <c r="F1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E2" t="s">
+        <v>14</v>
+      </c>
+      <c r="F2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3" t="s">
+        <v>9</v>
+      </c>
+      <c r="D3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C4" t="s">
+        <v>102</v>
+      </c>
+      <c r="D4" t="s">
+        <v>51</v>
+      </c>
+      <c r="E4" t="s">
+        <v>106</v>
+      </c>
+      <c r="F4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s">
+        <v>20</v>
+      </c>
+      <c r="B5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C5" t="s">
+        <v>107</v>
+      </c>
+      <c r="D5" t="s">
+        <v>41</v>
+      </c>
+      <c r="E5" t="s">
+        <v>108</v>
+      </c>
+      <c r="F5" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B6" t="s">
+        <v>23</v>
+      </c>
+      <c r="C6" t="s">
+        <v>108</v>
+      </c>
+      <c r="D6" t="s">
+        <v>62</v>
+      </c>
+      <c r="E6" t="s">
+        <v>59</v>
+      </c>
+      <c r="F6" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s">
+        <v>27</v>
+      </c>
+      <c r="B7" t="s">
+        <v>28</v>
+      </c>
+      <c r="C7" t="s">
+        <v>109</v>
+      </c>
+      <c r="D7" t="s">
+        <v>65</v>
+      </c>
+      <c r="E7" t="s">
+        <v>110</v>
+      </c>
+      <c r="F7" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s">
+        <v>29</v>
+      </c>
+      <c r="B8" t="s">
+        <v>30</v>
+      </c>
+      <c r="C8" t="s">
+        <v>111</v>
+      </c>
+      <c r="D8" t="s">
+        <v>112</v>
+      </c>
+      <c r="E8" t="s">
+        <v>63</v>
+      </c>
+      <c r="F8" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="s">
+        <v>34</v>
+      </c>
+      <c r="B12" t="s">
+        <v>9</v>
+      </c>
+      <c r="C12" t="s">
+        <v>9</v>
+      </c>
+      <c r="D12" t="s">
+        <v>9</v>
+      </c>
+      <c r="E12" t="s">
+        <v>9</v>
+      </c>
+      <c r="F12" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="s">
+        <v>35</v>
+      </c>
+      <c r="B32" t="s">
+        <v>36</v>
+      </c>
+      <c r="C32" t="s">
+        <v>37</v>
+      </c>
+      <c r="D32" t="s">
+        <v>37</v>
+      </c>
+      <c r="E32" t="s">
+        <v>37</v>
+      </c>
+      <c r="F32" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="s">
+        <v>38</v>
+      </c>
+      <c r="B33" t="s">
+        <v>39</v>
+      </c>
+      <c r="C33" t="s">
+        <v>31</v>
+      </c>
+      <c r="D33" t="s">
+        <v>113</v>
+      </c>
+      <c r="E33" t="s">
+        <v>114</v>
+      </c>
+      <c r="F33" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="s">
+        <v>71</v>
+      </c>
+      <c r="B42" t="s">
+        <v>9</v>
+      </c>
+      <c r="C42" t="s">
+        <v>9</v>
+      </c>
+      <c r="D42" t="s">
+        <v>9</v>
+      </c>
+      <c r="E42" t="s">
+        <v>9</v>
+      </c>
+      <c r="F42" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="s">
+        <v>72</v>
+      </c>
+      <c r="B43" t="s">
+        <v>73</v>
+      </c>
+      <c r="C43" t="s">
+        <v>115</v>
+      </c>
+      <c r="D43" t="s">
+        <v>46</v>
+      </c>
+      <c r="E43" t="s">
+        <v>115</v>
+      </c>
+      <c r="F43" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="s">
+        <v>76</v>
+      </c>
+      <c r="B56" t="s">
+        <v>77</v>
+      </c>
+      <c r="C56" t="s">
+        <v>116</v>
+      </c>
+      <c r="D56" t="s">
+        <v>46</v>
+      </c>
+      <c r="E56" t="s">
+        <v>116</v>
+      </c>
+      <c r="F56" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="s">
+        <v>79</v>
+      </c>
+      <c r="B57" t="s">
+        <v>80</v>
+      </c>
+      <c r="C57" t="s">
+        <v>116</v>
+      </c>
+      <c r="D57" t="s">
+        <v>46</v>
+      </c>
+      <c r="E57" t="s">
+        <v>116</v>
+      </c>
+      <c r="F57" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="s">
+        <v>81</v>
+      </c>
+      <c r="B58" t="s">
+        <v>77</v>
+      </c>
+      <c r="C58" t="s">
+        <v>116</v>
+      </c>
+      <c r="D58" t="s">
+        <v>46</v>
+      </c>
+      <c r="E58" t="s">
+        <v>116</v>
+      </c>
+      <c r="F58" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="s">
+        <v>43</v>
+      </c>
+      <c r="B67" t="s">
+        <v>9</v>
+      </c>
+      <c r="C67" t="s">
+        <v>9</v>
+      </c>
+      <c r="D67" t="s">
+        <v>9</v>
+      </c>
+      <c r="E67" t="s">
+        <v>9</v>
+      </c>
+      <c r="F67" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="s">
+        <v>44</v>
+      </c>
+      <c r="B68" t="s">
+        <v>43</v>
+      </c>
+      <c r="C68" t="s">
+        <v>117</v>
+      </c>
+      <c r="D68" t="s">
+        <v>46</v>
+      </c>
+      <c r="E68" t="s">
+        <v>117</v>
+      </c>
+      <c r="F68" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="s">
+        <v>82</v>
+      </c>
+      <c r="B69" t="s">
+        <v>9</v>
+      </c>
+      <c r="C69" t="s">
+        <v>9</v>
+      </c>
+      <c r="D69" t="s">
+        <v>9</v>
+      </c>
+      <c r="E69" t="s">
+        <v>9</v>
+      </c>
+      <c r="F69" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="s">
+        <v>83</v>
+      </c>
+      <c r="B70" t="s">
+        <v>84</v>
+      </c>
+      <c r="C70" t="s">
+        <v>118</v>
+      </c>
+      <c r="D70" t="s">
+        <v>51</v>
+      </c>
+      <c r="E70" t="s">
+        <v>119</v>
+      </c>
+      <c r="F70" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="s">
+        <v>87</v>
+      </c>
+      <c r="B79" t="s">
+        <v>88</v>
+      </c>
+      <c r="C79" t="s">
+        <v>37</v>
+      </c>
+      <c r="D79" t="s">
+        <v>37</v>
+      </c>
+      <c r="E79" t="s">
+        <v>37</v>
+      </c>
+      <c r="F79" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="s">
+        <v>89</v>
+      </c>
+      <c r="B80" t="s">
+        <v>90</v>
+      </c>
+      <c r="C80" t="s">
+        <v>120</v>
+      </c>
+      <c r="D80" t="s">
+        <v>46</v>
+      </c>
+      <c r="E80" t="s">
+        <v>120</v>
+      </c>
+      <c r="F80" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="s">
+        <v>93</v>
+      </c>
+      <c r="B81" t="s">
+        <v>94</v>
+      </c>
+      <c r="C81" t="s">
+        <v>120</v>
+      </c>
+      <c r="D81" t="s">
+        <v>46</v>
+      </c>
+      <c r="E81" t="s">
+        <v>120</v>
+      </c>
+      <c r="F81" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="s">
+        <v>95</v>
+      </c>
+      <c r="B101" t="s">
+        <v>96</v>
+      </c>
+      <c r="C101" t="s">
+        <v>121</v>
+      </c>
+      <c r="D101" t="s">
+        <v>46</v>
+      </c>
+      <c r="E101" t="s">
+        <v>121</v>
+      </c>
+      <c r="F101" t="s">
+        <v>92</v>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>122</v>
+      </c>
+      <c r="B1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C2" t="s">
+        <v>123</v>
+      </c>
+      <c r="D2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3" t="s">
+        <v>9</v>
+      </c>
+      <c r="D3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C4" t="s">
+        <v>124</v>
+      </c>
+      <c r="D4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s">
+        <v>20</v>
+      </c>
+      <c r="B5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C5" t="s">
+        <v>59</v>
+      </c>
+      <c r="D5" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B6" t="s">
+        <v>23</v>
+      </c>
+      <c r="C6" t="s">
+        <v>63</v>
+      </c>
+      <c r="D6" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s">
+        <v>27</v>
+      </c>
+      <c r="B7" t="s">
+        <v>28</v>
+      </c>
+      <c r="C7" t="s">
+        <v>68</v>
+      </c>
+      <c r="D7" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s">
+        <v>29</v>
+      </c>
+      <c r="B8" t="s">
+        <v>30</v>
+      </c>
+      <c r="C8" t="s">
+        <v>125</v>
+      </c>
+      <c r="D8" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="s">
+        <v>34</v>
+      </c>
+      <c r="B12" t="s">
+        <v>9</v>
+      </c>
+      <c r="C12" t="s">
+        <v>9</v>
+      </c>
+      <c r="D12" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="s">
+        <v>35</v>
+      </c>
+      <c r="B32" t="s">
+        <v>36</v>
+      </c>
+      <c r="C32" t="s">
+        <v>37</v>
+      </c>
+      <c r="D32" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="s">
+        <v>38</v>
+      </c>
+      <c r="B33" t="s">
+        <v>39</v>
+      </c>
+      <c r="C33" t="s">
+        <v>126</v>
+      </c>
+      <c r="D33" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="s">
+        <v>71</v>
+      </c>
+      <c r="B42" t="s">
+        <v>9</v>
+      </c>
+      <c r="C42" t="s">
+        <v>9</v>
+      </c>
+      <c r="D42" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="s">
+        <v>72</v>
+      </c>
+      <c r="B43" t="s">
+        <v>73</v>
+      </c>
+      <c r="C43" t="s">
+        <v>127</v>
+      </c>
+      <c r="D43" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="s">
+        <v>76</v>
+      </c>
+      <c r="B56" t="s">
+        <v>77</v>
+      </c>
+      <c r="C56" t="s">
+        <v>128</v>
+      </c>
+      <c r="D56" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="s">
+        <v>79</v>
+      </c>
+      <c r="B57" t="s">
+        <v>80</v>
+      </c>
+      <c r="C57" t="s">
+        <v>128</v>
+      </c>
+      <c r="D57" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="s">
+        <v>81</v>
+      </c>
+      <c r="B58" t="s">
+        <v>77</v>
+      </c>
+      <c r="C58" t="s">
+        <v>128</v>
+      </c>
+      <c r="D58" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="s">
+        <v>43</v>
+      </c>
+      <c r="B67" t="s">
+        <v>9</v>
+      </c>
+      <c r="C67" t="s">
+        <v>9</v>
+      </c>
+      <c r="D67" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="s">
+        <v>44</v>
+      </c>
+      <c r="B68" t="s">
+        <v>43</v>
+      </c>
+      <c r="C68" t="s">
+        <v>129</v>
+      </c>
+      <c r="D68" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="s">
+        <v>82</v>
+      </c>
+      <c r="B69" t="s">
+        <v>9</v>
+      </c>
+      <c r="C69" t="s">
+        <v>9</v>
+      </c>
+      <c r="D69" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="s">
+        <v>83</v>
+      </c>
+      <c r="B70" t="s">
+        <v>84</v>
+      </c>
+      <c r="C70" t="s">
+        <v>130</v>
+      </c>
+      <c r="D70" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="s">
+        <v>87</v>
+      </c>
+      <c r="B79" t="s">
+        <v>88</v>
+      </c>
+      <c r="C79" t="s">
+        <v>37</v>
+      </c>
+      <c r="D79" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="s">
+        <v>89</v>
+      </c>
+      <c r="B80" t="s">
+        <v>90</v>
+      </c>
+      <c r="C80" t="s">
+        <v>131</v>
+      </c>
+      <c r="D80" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="s">
+        <v>93</v>
+      </c>
+      <c r="B81" t="s">
+        <v>94</v>
+      </c>
+      <c r="C81" t="s">
+        <v>131</v>
+      </c>
+      <c r="D81" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="s">
+        <v>95</v>
+      </c>
+      <c r="B101" t="s">
+        <v>96</v>
+      </c>
+      <c r="C101" t="s">
+        <v>132</v>
+      </c>
+      <c r="D101" t="s">
+        <v>92</v>
       </c>
     </row>
   </sheetData>

</xml_diff>